<commit_message>
Auto update: scraping + analisis 2026-09-16 02:31 WIB
</commit_message>
<xml_diff>
--- a/data/output/distribusi_topik.xlsx
+++ b/data/output/distribusi_topik.xlsx
@@ -433,7 +433,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>1032</v>
+        <v>1942</v>
       </c>
     </row>
     <row r="3">
@@ -441,7 +441,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>946</v>
+        <v>296</v>
       </c>
     </row>
     <row r="4">
@@ -449,7 +449,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>790</v>
+        <v>219</v>
       </c>
     </row>
     <row r="5">
@@ -457,7 +457,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>264</v>
+        <v>1836</v>
       </c>
     </row>
     <row r="6">
@@ -465,7 +465,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>1848</v>
+        <v>709</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: scraping + analisis 2026-09-22 02:50 WIB
</commit_message>
<xml_diff>
--- a/data/output/distribusi_topik.xlsx
+++ b/data/output/distribusi_topik.xlsx
@@ -433,7 +433,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>1942</v>
+        <v>1943</v>
       </c>
     </row>
     <row r="3">
@@ -441,7 +441,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>296</v>
+        <v>297</v>
       </c>
     </row>
     <row r="4">
@@ -449,7 +449,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>219</v>
+        <v>223</v>
       </c>
     </row>
     <row r="5">
@@ -457,7 +457,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>1836</v>
+        <v>1817</v>
       </c>
     </row>
     <row r="6">
@@ -465,7 +465,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>709</v>
+        <v>725</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: scraping + analisis 2026-09-24 02:32 WIB
</commit_message>
<xml_diff>
--- a/data/output/distribusi_topik.xlsx
+++ b/data/output/distribusi_topik.xlsx
@@ -433,7 +433,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>1943</v>
+        <v>2056</v>
       </c>
     </row>
     <row r="3">
@@ -441,7 +441,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>297</v>
+        <v>555</v>
       </c>
     </row>
     <row r="4">
@@ -449,7 +449,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>223</v>
+        <v>256</v>
       </c>
     </row>
     <row r="5">
@@ -457,7 +457,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>1817</v>
+        <v>1910</v>
       </c>
     </row>
     <row r="6">
@@ -465,7 +465,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>725</v>
+        <v>277</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: scraping + analisis 2026-09-25 02:33 WIB
</commit_message>
<xml_diff>
--- a/data/output/distribusi_topik.xlsx
+++ b/data/output/distribusi_topik.xlsx
@@ -433,7 +433,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>2056</v>
+        <v>2059</v>
       </c>
     </row>
     <row r="3">
@@ -441,7 +441,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>555</v>
+        <v>552</v>
       </c>
     </row>
     <row r="4">
@@ -449,7 +449,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>256</v>
+        <v>251</v>
       </c>
     </row>
     <row r="5">
@@ -457,7 +457,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>1910</v>
+        <v>1920</v>
       </c>
     </row>
     <row r="6">
@@ -465,7 +465,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>277</v>
+        <v>273</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: scraping + analisis 2026-10-01 03:18 WIB
</commit_message>
<xml_diff>
--- a/data/output/distribusi_topik.xlsx
+++ b/data/output/distribusi_topik.xlsx
@@ -433,7 +433,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>2059</v>
+        <v>578</v>
       </c>
     </row>
     <row r="3">
@@ -441,7 +441,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>552</v>
+        <v>1553</v>
       </c>
     </row>
     <row r="4">
@@ -449,7 +449,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>251</v>
+        <v>288</v>
       </c>
     </row>
     <row r="5">
@@ -457,7 +457,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>1920</v>
+        <v>2530</v>
       </c>
     </row>
     <row r="6">
@@ -465,7 +465,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>273</v>
+        <v>166</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: scraping + analisis 2026-10-03 03:09 WIB
</commit_message>
<xml_diff>
--- a/data/output/distribusi_topik.xlsx
+++ b/data/output/distribusi_topik.xlsx
@@ -433,7 +433,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>578</v>
+        <v>1923</v>
       </c>
     </row>
     <row r="3">
@@ -441,7 +441,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>1553</v>
+        <v>282</v>
       </c>
     </row>
     <row r="4">
@@ -449,7 +449,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>288</v>
+        <v>224</v>
       </c>
     </row>
     <row r="5">
@@ -457,7 +457,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>2530</v>
+        <v>2127</v>
       </c>
     </row>
     <row r="6">
@@ -465,7 +465,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>166</v>
+        <v>589</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: scraping + analisis 2026-10-04 03:48 WIB
</commit_message>
<xml_diff>
--- a/data/output/distribusi_topik.xlsx
+++ b/data/output/distribusi_topik.xlsx
@@ -433,7 +433,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>1923</v>
+        <v>1926</v>
       </c>
     </row>
     <row r="3">
@@ -441,7 +441,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>282</v>
+        <v>287</v>
       </c>
     </row>
     <row r="4">
@@ -449,7 +449,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>224</v>
+        <v>222</v>
       </c>
     </row>
     <row r="5">
@@ -457,7 +457,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>2127</v>
+        <v>2126</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
Auto update: scraping + analisis 2026-10-07 03:32 WIB
</commit_message>
<xml_diff>
--- a/data/output/distribusi_topik.xlsx
+++ b/data/output/distribusi_topik.xlsx
@@ -433,7 +433,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>1926</v>
+        <v>2008</v>
       </c>
     </row>
     <row r="3">
@@ -441,7 +441,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>287</v>
+        <v>235</v>
       </c>
     </row>
     <row r="4">
@@ -449,7 +449,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>222</v>
+        <v>184</v>
       </c>
     </row>
     <row r="5">
@@ -457,7 +457,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>2126</v>
+        <v>207</v>
       </c>
     </row>
     <row r="6">
@@ -465,7 +465,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>589</v>
+        <v>2530</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto update: scraping + analisis 2026-10-28 03:18 WIB
</commit_message>
<xml_diff>
--- a/data/output/distribusi_topik.xlsx
+++ b/data/output/distribusi_topik.xlsx
@@ -433,7 +433,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>2008</v>
+        <v>2013</v>
       </c>
     </row>
     <row r="3">
@@ -441,7 +441,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="4">
@@ -449,7 +449,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>184</v>
+        <v>181</v>
       </c>
     </row>
     <row r="5">
@@ -457,7 +457,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>207</v>
+        <v>209</v>
       </c>
     </row>
     <row r="6">
@@ -465,7 +465,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>2530</v>
+        <v>2526</v>
       </c>
     </row>
   </sheetData>

</xml_diff>